<commit_message>
Make Exception Workbook English-first with a Thai locale.
Add /th/ routing, global English samples, safer date formats, broader currency parsing, and SEO copy while keeping the reference-and-amount matching engine unchanged.
</commit_message>
<xml_diff>
--- a/public/sample-orders.xlsx
+++ b/public/sample-orders.xlsx
@@ -401,30 +401,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>เลขที่ใบสั่ง</v>
+        <v>Order ID</v>
       </c>
       <c r="B1" t="str">
-        <v>ลูกค้า</v>
+        <v>Customer</v>
       </c>
       <c r="C1" t="str">
-        <v>ยอดเงิน</v>
+        <v>Amount</v>
       </c>
       <c r="D1" t="str">
-        <v>วันที่</v>
+        <v>Date</v>
       </c>
       <c r="E1" t="str">
-        <v>ช่องทาง</v>
+        <v>Channel</v>
       </c>
       <c r="F1" t="str">
-        <v>บันทึก</v>
+        <v>Note</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v xml:space="preserve">ORD-24001 </v>
+        <v xml:space="preserve">ORD-1001 </v>
       </c>
       <c r="B2" t="str">
-        <v>หจก. นภาวัสดุ</v>
+        <v>Alex Smith</v>
       </c>
       <c r="C2">
         <v>1000</v>
@@ -433,18 +433,18 @@
         <v>2026-02-01</v>
       </c>
       <c r="E2" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F2" t="str">
-        <v>ช่องว่างท้ายเลขที่</v>
+        <v>trailing space on reference</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ORD-24002</v>
+        <v>ORD-1002</v>
       </c>
       <c r="B3" t="str">
-        <v>บริษัท บ้านสวนบรรจุภัณฑ์ จำกัด</v>
+        <v>Jordan Lee</v>
       </c>
       <c r="C3">
         <v>1075.5</v>
@@ -453,7 +453,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E3" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -461,10 +461,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ORD 24003</v>
+        <v>ORD 1003</v>
       </c>
       <c r="B4" t="str">
-        <v>ร้าน พีระอะไหล่</v>
+        <v>Sam Rivera</v>
       </c>
       <c r="C4">
         <v>1151</v>
@@ -473,7 +473,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E4" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ORD-24004</v>
+        <v>ORD-1004</v>
       </c>
       <c r="B5" t="str">
-        <v>บริษัท ลานนาเกษตร จำกัด</v>
+        <v>Casey Morgan</v>
       </c>
       <c r="C5">
         <v>1225</v>
@@ -493,7 +493,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E5" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -501,10 +501,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ORD-24005</v>
+        <v>ORD-1005</v>
       </c>
       <c r="B6" t="str">
-        <v>หจก. ท่าเรือบรรทุก</v>
+        <v>Riley Chen</v>
       </c>
       <c r="C6">
         <v>1300.5</v>
@@ -513,7 +513,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E6" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -521,10 +521,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ORD-24006</v>
+        <v>ORD-1006</v>
       </c>
       <c r="B7" t="str">
-        <v>ร้าน สมชายการช่าง</v>
+        <v>Avery Brooks</v>
       </c>
       <c r="C7">
         <v>1376</v>
@@ -533,7 +533,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E7" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -541,10 +541,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v xml:space="preserve">ORD-24007 </v>
+        <v xml:space="preserve">ORD-1007 </v>
       </c>
       <c r="B8" t="str">
-        <v>บริษัท ตะวันออกพลาสติก จำกัด</v>
+        <v>Quinn Patel</v>
       </c>
       <c r="C8">
         <v>1450</v>
@@ -553,7 +553,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E8" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -561,10 +561,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ORD-24008</v>
+        <v>ORD-1008</v>
       </c>
       <c r="B9" t="str">
-        <v>หจก. เชียงรายอาหารแห้ง</v>
+        <v>Jamie Nguyen</v>
       </c>
       <c r="C9">
         <v>1525.5</v>
@@ -573,7 +573,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E9" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -581,10 +581,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ORD 24009</v>
+        <v>ORD 1009</v>
       </c>
       <c r="B10" t="str">
-        <v>ร้าน วงศ์สว่างไฟฟ้า</v>
+        <v>Taylor Kim</v>
       </c>
       <c r="C10">
         <v>1601</v>
@@ -593,7 +593,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E10" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -601,10 +601,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ORD-24010</v>
+        <v>ORD-1010</v>
       </c>
       <c r="B11" t="str">
-        <v>บริษัท แม่กลองประมง จำกัด</v>
+        <v>Morgan Diaz</v>
       </c>
       <c r="C11">
         <v>1675</v>
@@ -613,7 +613,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E11" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -621,10 +621,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ORD-24011</v>
+        <v>ORD-1011</v>
       </c>
       <c r="B12" t="str">
-        <v>หจก. ปากน้ำขนส่ง</v>
+        <v>Cameron Ortiz</v>
       </c>
       <c r="C12">
         <v>1750.5</v>
@@ -633,7 +633,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E12" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -641,10 +641,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ORD-24012</v>
+        <v>ORD-1012</v>
       </c>
       <c r="B13" t="str">
-        <v>ร้าน อรุณเครื่องเขียน</v>
+        <v>Drew Santos</v>
       </c>
       <c r="C13">
         <v>1826</v>
@@ -653,7 +653,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E13" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -661,10 +661,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">ORD-24013 </v>
+        <v xml:space="preserve">ORD-1013 </v>
       </c>
       <c r="B14" t="str">
-        <v>หจก. นภาวัสดุ</v>
+        <v>Alex Smith</v>
       </c>
       <c r="C14">
         <v>1900</v>
@@ -673,7 +673,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E14" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -681,10 +681,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ORD-24014</v>
+        <v>ORD-1014</v>
       </c>
       <c r="B15" t="str">
-        <v>บริษัท บ้านสวนบรรจุภัณฑ์ จำกัด</v>
+        <v>Jordan Lee</v>
       </c>
       <c r="C15">
         <v>1975.5</v>
@@ -693,7 +693,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E15" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -701,10 +701,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ORD 24015</v>
+        <v>ORD 1015</v>
       </c>
       <c r="B16" t="str">
-        <v>ร้าน พีระอะไหล่</v>
+        <v>Sam Rivera</v>
       </c>
       <c r="C16">
         <v>2051</v>
@@ -713,7 +713,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E16" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -721,10 +721,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ORD-24016</v>
+        <v>ORD-1016</v>
       </c>
       <c r="B17" t="str">
-        <v>บริษัท ลานนาเกษตร จำกัด</v>
+        <v>Casey Morgan</v>
       </c>
       <c r="C17">
         <v>2125</v>
@@ -733,7 +733,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E17" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -741,10 +741,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ORD-24017</v>
+        <v>ORD-1017</v>
       </c>
       <c r="B18" t="str">
-        <v>หจก. ท่าเรือบรรทุก</v>
+        <v>Riley Chen</v>
       </c>
       <c r="C18">
         <v>2200.5</v>
@@ -753,7 +753,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E18" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -761,10 +761,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ORD-24018</v>
+        <v>ORD-1018</v>
       </c>
       <c r="B19" t="str">
-        <v>ร้าน สมชายการช่าง</v>
+        <v>Avery Brooks</v>
       </c>
       <c r="C19">
         <v>2276</v>
@@ -773,7 +773,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E19" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -781,10 +781,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">ORD-24019 </v>
+        <v xml:space="preserve">ORD-1019 </v>
       </c>
       <c r="B20" t="str">
-        <v>บริษัท ตะวันออกพลาสติก จำกัด</v>
+        <v>Quinn Patel</v>
       </c>
       <c r="C20">
         <v>2350</v>
@@ -793,7 +793,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E20" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -801,10 +801,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ORD-24020</v>
+        <v>ORD-1020</v>
       </c>
       <c r="B21" t="str">
-        <v>หจก. เชียงรายอาหารแห้ง</v>
+        <v>Jamie Nguyen</v>
       </c>
       <c r="C21">
         <v>2425.5</v>
@@ -813,7 +813,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E21" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -821,10 +821,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ORD 24021</v>
+        <v>ORD 1021</v>
       </c>
       <c r="B22" t="str">
-        <v>ร้าน วงศ์สว่างไฟฟ้า</v>
+        <v>Taylor Kim</v>
       </c>
       <c r="C22">
         <v>2501</v>
@@ -833,7 +833,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E22" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -841,10 +841,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ORD-24022</v>
+        <v>ORD-1022</v>
       </c>
       <c r="B23" t="str">
-        <v>บริษัท แม่กลองประมง จำกัด</v>
+        <v>Morgan Diaz</v>
       </c>
       <c r="C23">
         <v>2575</v>
@@ -853,7 +853,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E23" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -861,10 +861,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ORD-24023</v>
+        <v>ORD-1023</v>
       </c>
       <c r="B24" t="str">
-        <v>หจก. ปากน้ำขนส่ง</v>
+        <v>Cameron Ortiz</v>
       </c>
       <c r="C24">
         <v>2650.5</v>
@@ -873,7 +873,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E24" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F24" t="str">
         <v/>
@@ -881,10 +881,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ORD-24024</v>
+        <v>ORD-1024</v>
       </c>
       <c r="B25" t="str">
-        <v>ร้าน อรุณเครื่องเขียน</v>
+        <v>Drew Santos</v>
       </c>
       <c r="C25">
         <v>2726</v>
@@ -893,7 +893,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E25" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F25" t="str">
         <v/>
@@ -901,10 +901,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">ORD-24025 </v>
+        <v xml:space="preserve">ORD-1025 </v>
       </c>
       <c r="B26" t="str">
-        <v>หจก. นภาวัสดุ</v>
+        <v>Alex Smith</v>
       </c>
       <c r="C26">
         <v>2800</v>
@@ -913,7 +913,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E26" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F26" t="str">
         <v/>
@@ -921,10 +921,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ORD-24026</v>
+        <v>ORD-1026</v>
       </c>
       <c r="B27" t="str">
-        <v>บริษัท บ้านสวนบรรจุภัณฑ์ จำกัด</v>
+        <v>Jordan Lee</v>
       </c>
       <c r="C27">
         <v>2875.5</v>
@@ -933,7 +933,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E27" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -941,10 +941,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ORD 24027</v>
+        <v>ORD 1027</v>
       </c>
       <c r="B28" t="str">
-        <v>ร้าน พีระอะไหล่</v>
+        <v>Sam Rivera</v>
       </c>
       <c r="C28">
         <v>2951</v>
@@ -953,7 +953,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E28" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -961,10 +961,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ORD-24028</v>
+        <v>ORD-1028</v>
       </c>
       <c r="B29" t="str">
-        <v>บริษัท ลานนาเกษตร จำกัด</v>
+        <v>Casey Morgan</v>
       </c>
       <c r="C29">
         <v>3025</v>
@@ -973,7 +973,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E29" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F29" t="str">
         <v/>
@@ -981,10 +981,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ORD-24029</v>
+        <v>ORD-1029</v>
       </c>
       <c r="B30" t="str">
-        <v>หจก. ท่าเรือบรรทุก</v>
+        <v>Riley Chen</v>
       </c>
       <c r="C30">
         <v>3100.5</v>
@@ -993,7 +993,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E30" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F30" t="str">
         <v/>
@@ -1001,10 +1001,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ORD-24030</v>
+        <v>ORD-1030</v>
       </c>
       <c r="B31" t="str">
-        <v>ร้าน สมชายการช่าง</v>
+        <v>Avery Brooks</v>
       </c>
       <c r="C31">
         <v>3176</v>
@@ -1013,7 +1013,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="E31" t="str">
-        <v>เงินสด</v>
+        <v>Transfer</v>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -1021,10 +1021,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ORD-24101</v>
+        <v>ORD-1101</v>
       </c>
       <c r="B32" t="str">
-        <v>หจก. นภาวัสดุ</v>
+        <v>Alex Smith</v>
       </c>
       <c r="C32">
         <v>10000</v>
@@ -1033,7 +1033,7 @@
         <v>2026-03-20</v>
       </c>
       <c r="E32" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F32" t="str">
         <v/>
@@ -1041,10 +1041,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ORD-24102</v>
+        <v>ORD-1102</v>
       </c>
       <c r="B33" t="str">
-        <v>บริษัท บ้านสวนบรรจุภัณฑ์ จำกัด</v>
+        <v>Jordan Lee</v>
       </c>
       <c r="C33">
         <v>2500.5</v>
@@ -1053,7 +1053,7 @@
         <v>2026-03-20</v>
       </c>
       <c r="E33" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F33" t="str">
         <v/>
@@ -1061,10 +1061,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ORD-24103</v>
+        <v>ORD-1103</v>
       </c>
       <c r="B34" t="str">
-        <v>ร้าน พีระอะไหล่</v>
+        <v>Sam Rivera</v>
       </c>
       <c r="C34" t="str">
         <v xml:space="preserve"> 1,500.00 </v>
@@ -1073,7 +1073,7 @@
         <v>2026-03-20</v>
       </c>
       <c r="E34" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F34" t="str">
         <v/>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ORD-24104</v>
+        <v>ORD-1104</v>
       </c>
       <c r="B35" t="str">
-        <v>บริษัท ลานนาเกษตร จำกัด</v>
+        <v>Casey Morgan</v>
       </c>
       <c r="C35">
         <v>800</v>
@@ -1093,7 +1093,7 @@
         <v>2026-03-20</v>
       </c>
       <c r="E35" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -1101,10 +1101,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ORD-24105</v>
+        <v>ORD-1105</v>
       </c>
       <c r="B36" t="str">
-        <v>หจก. ท่าเรือบรรทุก</v>
+        <v>Riley Chen</v>
       </c>
       <c r="C36">
         <v>4200</v>
@@ -1113,7 +1113,7 @@
         <v>2026-03-20</v>
       </c>
       <c r="E36" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F36" t="str">
         <v/>
@@ -1121,19 +1121,19 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ORD-24106</v>
+        <v>ORD-1106</v>
       </c>
       <c r="B37" t="str">
-        <v>ร้าน สมชายการช่าง</v>
+        <v>Avery Brooks</v>
       </c>
       <c r="C37" t="str">
-        <v>฿3,300.00</v>
+        <v>$3,300.00</v>
       </c>
       <c r="D37" t="str">
         <v>2026-03-20</v>
       </c>
       <c r="E37" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1141,10 +1141,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ORD-24201</v>
+        <v>ORD-1201</v>
       </c>
       <c r="B38" t="str">
-        <v>หจก. นภาวัสดุ</v>
+        <v>Alex Smith</v>
       </c>
       <c r="C38">
         <v>2100</v>
@@ -1153,18 +1153,18 @@
         <v>2026-04-02</v>
       </c>
       <c r="E38" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F38" t="str">
-        <v>ค้างในไฟล์ใบสั่ง</v>
+        <v>only in file A</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ORD-24202</v>
+        <v>ORD-1202</v>
       </c>
       <c r="B39" t="str">
-        <v>บริษัท บ้านสวนบรรจุภัณฑ์ จำกัด</v>
+        <v>Jordan Lee</v>
       </c>
       <c r="C39">
         <v>2110</v>
@@ -1173,7 +1173,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E39" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -1181,10 +1181,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ORD-24203</v>
+        <v>ORD-1203</v>
       </c>
       <c r="B40" t="str">
-        <v>ร้าน พีระอะไหล่</v>
+        <v>Sam Rivera</v>
       </c>
       <c r="C40">
         <v>2120</v>
@@ -1193,7 +1193,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E40" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -1201,10 +1201,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ORD-24204</v>
+        <v>ORD-1204</v>
       </c>
       <c r="B41" t="str">
-        <v>บริษัท ลานนาเกษตร จำกัด</v>
+        <v>Casey Morgan</v>
       </c>
       <c r="C41">
         <v>2130</v>
@@ -1213,7 +1213,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E41" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F41" t="str">
         <v/>
@@ -1221,10 +1221,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ORD-24205</v>
+        <v>ORD-1205</v>
       </c>
       <c r="B42" t="str">
-        <v>หจก. ท่าเรือบรรทุก</v>
+        <v>Riley Chen</v>
       </c>
       <c r="C42">
         <v>2140</v>
@@ -1233,7 +1233,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E42" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1241,10 +1241,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ORD-24206</v>
+        <v>ORD-1206</v>
       </c>
       <c r="B43" t="str">
-        <v>ร้าน สมชายการช่าง</v>
+        <v>Avery Brooks</v>
       </c>
       <c r="C43">
         <v>2150</v>
@@ -1253,7 +1253,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E43" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F43" t="str">
         <v/>
@@ -1261,10 +1261,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ORD-24207</v>
+        <v>ORD-1207</v>
       </c>
       <c r="B44" t="str">
-        <v>บริษัท ตะวันออกพลาสติก จำกัด</v>
+        <v>Quinn Patel</v>
       </c>
       <c r="C44">
         <v>2160</v>
@@ -1273,7 +1273,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E44" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -1281,10 +1281,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ORD-24208</v>
+        <v>ORD-1208</v>
       </c>
       <c r="B45" t="str">
-        <v>หจก. เชียงรายอาหารแห้ง</v>
+        <v>Jamie Nguyen</v>
       </c>
       <c r="C45">
         <v>2170</v>
@@ -1293,7 +1293,7 @@
         <v>2026-04-02</v>
       </c>
       <c r="E45" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -1301,10 +1301,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ORD-24401</v>
+        <v>ORD-1401</v>
       </c>
       <c r="B46" t="str">
-        <v>หจก. นภาวัสดุ</v>
+        <v>Alex Smith</v>
       </c>
       <c r="C46">
         <v>500</v>
@@ -1313,7 +1313,7 @@
         <v>2026-04-08</v>
       </c>
       <c r="E46" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Card</v>
       </c>
       <c r="F46" t="str">
         <v/>
@@ -1321,10 +1321,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ord 24401</v>
+        <v>ord 1401</v>
       </c>
       <c r="B47" t="str">
-        <v>บริษัท บ้านสวนบรรจุภัณฑ์ จำกัด</v>
+        <v>Jordan Lee</v>
       </c>
       <c r="C47">
         <v>640</v>
@@ -1333,7 +1333,7 @@
         <v>2026-04-08</v>
       </c>
       <c r="E47" t="str">
-        <v>เงินสด</v>
+        <v>Cash</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -1341,10 +1341,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ORD-24402</v>
+        <v>ORD-1402</v>
       </c>
       <c r="B48" t="str">
-        <v>ร้าน พีระอะไหล่</v>
+        <v>Sam Rivera</v>
       </c>
       <c r="C48">
         <v>900</v>
@@ -1353,7 +1353,7 @@
         <v>2026-04-09</v>
       </c>
       <c r="E48" t="str">
-        <v>โอนธนาคาร</v>
+        <v>Transfer</v>
       </c>
       <c r="F48" t="str">
         <v/>

</xml_diff>